<commit_message>
Apply Rule 804 to latest Farda export retaining full bundle contents and source quantities
</commit_message>
<xml_diff>
--- a/catalog-files/Farda_Foods_Professional.xlsx
+++ b/catalog-files/Farda_Foods_Professional.xlsx
@@ -1868,6 +1868,7 @@
 • Malai Boti Masala
 • Salt
 • Garlic Powder
+• Ginger Powder
 • Garam Masala Powder</t>
         </is>
       </c>
@@ -1943,6 +1944,8 @@
 • White Qorma Masala
 • Salt
 • Coriander Seeds
+• Garlic Powder
+• Ginger Powder
 • Garam Masala Powder</t>
         </is>
       </c>
@@ -2018,6 +2021,10 @@
 • Seekh kabab Masala
 • Salt
 • Turmeric Powder
+• Coriander Powder
+• Red Chilli Powder
+• Garlic Powder
+• Ginger Powder
 • Garam Masala Powder</t>
         </is>
       </c>
@@ -2092,6 +2099,11 @@
 Bundle contents:
 • Chicken Tikka Masala
 • Salt
+• Turmeric Powder
+• Coriander Powder
+• Red Chilli Powder
+• Garlic Powder
+• Ginger Powder
 • Garam Masala Powder
 • Chaat Masala Powder</t>
         </is>
@@ -2168,7 +2180,12 @@
 • Achar Gosht Masala
 • Salt
 • Turmeric Powder
-• Garam Masala Powder</t>
+• Coriander Powder
+• Red Chilli Powder
+• Garlic Powder
+• Ginger Powder
+• Garam Masala Powder
+• Cumin Powder</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -2243,7 +2260,12 @@
 • Karahi Masala
 • Salt
 • Turmeric Powder
-• Garam Masala Powder</t>
+• Coriander Powder
+• Red Chilli Powder
+• Garlic Powder
+• Ginger Powder
+• Garam Masala Powder
+• Cumin Powder</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -2318,7 +2340,12 @@
 • Qorma Masala
 • Salt
 • Turmeric Powder
-• Garam Masala Powder</t>
+• Coriander Powder
+• Red Chilli Powder
+• Garlic Powder
+• Ginger Powder
+• Garam Masala Powder
+• Cumin Powder</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -2393,6 +2420,10 @@
 • Biryani Masala
 • Salt
 • Turmeric Powder
+• Coriander Powder
+• Red Chilli Powder
+• Garlic Powder
+• Ginger Powder
 • Garam Masala Sabit</t>
         </is>
       </c>
@@ -2468,6 +2499,10 @@
 • Bombay Biryani Masala
 • Salt
 • Turmeric Powder
+• Coriander Powder
+• Red Chilli Powder
+• Garlic Powder
+• Ginger Powder
 • Garam Masala Sabit</t>
         </is>
       </c>
@@ -2681,7 +2716,8 @@
       <c r="E13" t="inlineStr">
         <is>
           <t xml:space="preserve">Farda straight vermicelli, made from wheat.
-Pack size: 350 g.</t>
+Pack size: 350 g.
+Uses: sweet and savoury recipes.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -2823,7 +2859,8 @@
       <c r="E15" t="inlineStr">
         <is>
           <t xml:space="preserve">Farda Garam Masalah is a spice blend for everyday cooking.
-Pack size: 50 g.</t>
+Pack size: 50 g.
+Ingredients (as listed): cinnamon, peppercorns, cardamom, mustard seeds, coriander seeds, cloves, mace, and nutmeg.</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -3036,7 +3073,8 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Farda Chaat Masala is a spice blend for chaat and savoury snacks.</t>
+          <t xml:space="preserve">Farda Chaat Masala is a spice blend for chaat and savoury snacks.
+Available pack sizes: 50 g, 100 g.</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -3111,7 +3149,8 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Farda cumin powder, made from ground cumin seeds, for cooking and spice blends.</t>
+          <t xml:space="preserve">Farda cumin powder, made from ground cumin seeds, for cooking and spice blends.
+Pack size: 50 g.</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -3181,7 +3220,8 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Farda garlic powder, a ground seasoning for cooking.</t>
+          <t xml:space="preserve">Farda garlic powder, a ground seasoning for cooking.
+Pack size: 50 g.</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -3251,7 +3291,8 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Farda coriander powder, a ground spice for cooking.</t>
+          <t xml:space="preserve">Farda coriander powder, a ground spice for cooking.
+Pack size: 100 g.</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -3321,7 +3362,8 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Farda turmeric powder for adding colour and flavour to food.</t>
+          <t xml:space="preserve">Farda turmeric powder for adding colour and flavour to food.
+Available pack sizes: 50 g, 100 g.</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -3392,7 +3434,7 @@
       <c r="E23" t="inlineStr">
         <is>
           <t xml:space="preserve">Farda red chilli powder for adding chilli flavour to food.
-Available pack sizes: 100 g and 200 g.</t>
+Available pack sizes: 100 g, 200 g.</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -3467,7 +3509,8 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Farda ground black pepper for seasoning and cooking.</t>
+          <t xml:space="preserve">Farda ground black pepper for seasoning and cooking.
+Pack size: 50 g.</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -3537,7 +3580,8 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Farda white cumin seeds for cooking and spice blends.</t>
+          <t xml:space="preserve">Farda white cumin seeds for cooking and spice blends.
+Pack size: 100 g.</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -3607,7 +3651,9 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Farda Garam Masala Saabit is a whole-spice blend for Pakistani cooking. The blend includes cloves, cinnamon, cardamom, cumin, coriander, nutmeg, bay leaf, mace and black pepper.</t>
+          <t xml:space="preserve">Farda Garam Masala Saabit is a whole-spice blend for Pakistani cooking.
+Pack size: 100 g.
+Ingredients (as listed): cloves, cinnamon, cardamoms, cumin, coriander, nutmeg, bay leaf, mace and black pepper.</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -3820,7 +3866,8 @@
       <c r="E29" t="inlineStr">
         <is>
           <t xml:space="preserve">Farda Garam Masala Powder is a spice blend for everyday cooking.
-Pack quantity: 12.</t>
+Pack quantity: 12.
+Ingredients (as listed): cinnamon, peppercorns, cardamom, mustard seeds, coriander seeds, cloves, mace, and nutmeg.</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -4034,7 +4081,8 @@
         <is>
           <t xml:space="preserve">Farda Achar Gosht is a spice blend for achar gosht.
 Pack quantity: 12.
-Unit weight: 12 g.</t>
+Unit weight: 12 g.
+Flavour: tangy and spicy, with a pickle-style taste.</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -4106,7 +4154,8 @@
         <is>
           <t xml:space="preserve">Farda Biryani Masala is a spice blend for biryani.
 Pack quantity: 12.
-Unit weight: 12 g.</t>
+Unit weight: 12 g.
+Flavour notes: mild spice with red chilli and saffron.</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -4178,7 +4227,8 @@
         <is>
           <t xml:space="preserve">Farda Karahi Gosht is a spice blend for karahi dishes.
 Pack quantity: 12.
-Unit weight: 12 g.</t>
+Unit weight: 12 g.
+Ingredients (as listed): cumin, coriander, ginger, garlic, turmeric, and red chili powder.</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -4322,7 +4372,8 @@
         <is>
           <t xml:space="preserve">Farda Achar Gosht is a spice blend for achar gosht.
 Pack quantity: 12.
-Unit weight: 21 g.</t>
+Unit weight: 21 g.
+Flavour: tangy and spicy, with a pickle-style taste.</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -4394,7 +4445,8 @@
         <is>
           <t xml:space="preserve">Farda Biryani Masala is a spice blend for biryani.
 Pack quantity: 12.
-Unit weight: 21 g.</t>
+Unit weight: 21 g.
+Flavour notes: mild spice with red chilli and saffron.</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -4466,7 +4518,8 @@
         <is>
           <t xml:space="preserve">Farda Karahi Gosht is a spice blend for karahi dishes.
 Pack quantity: 12.
-Unit weight: 21 g.</t>
+Unit weight: 21 g.
+Ingredients (as listed): cumin, coriander, ginger, garlic, turmeric, and red chili powder.</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -4609,7 +4662,8 @@
       <c r="E40" t="inlineStr">
         <is>
           <t xml:space="preserve">Farda Achar Gosht Masala is a spice blend for achar gosht.
-Pack size: 50 g.</t>
+Pack size: 50 g.
+Flavour: tangy and spicy, with a pickle-style taste.</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -4680,7 +4734,8 @@
       <c r="E41" t="inlineStr">
         <is>
           <t xml:space="preserve">Farda Bombay Biryani Masala is a spice blend for Bombay biryani.
-Pack size: 50 g.</t>
+Pack size: 50 g.
+Ingredients (as listed): Turmeric, Coriander Powder, Star anise, Carom seeds, Mango powder, Cinnamomum Tamala, Cloves with the hint of Red chili powder.</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -4822,7 +4877,8 @@
       <c r="E43" t="inlineStr">
         <is>
           <t xml:space="preserve">Farda Karahi Masala is a spice blend for karahi dishes.
-Pack size: 50 g.</t>
+Pack size: 50 g.
+Ingredients (as listed): cumin, coriander, ginger, garlic, turmeric, and red chili powder.</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -5105,7 +5161,8 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Farda refined white salt, fortified with iodine, for everyday seasoning.</t>
+          <t xml:space="preserve">Farda refined white salt, fortified with iodine, for everyday seasoning.
+Pack size: 800 g.</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -5175,7 +5232,8 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Farda iodized refined Himalayan pink salt for everyday seasoning.</t>
+          <t xml:space="preserve">Farda iodized refined Himalayan pink salt for everyday seasoning.
+Pack size: 800 g.</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -5245,7 +5303,8 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Farda ginger powder, a ground seasoning for cooking.</t>
+          <t xml:space="preserve">Farda ginger powder, a ground seasoning for cooking.
+Pack size: 50 g.</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -5315,7 +5374,8 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Farda whole black pepper for seasoning and cooking.</t>
+          <t xml:space="preserve">Farda whole black pepper for seasoning and cooking.
+Pack size: 100 g.</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -5386,7 +5446,8 @@
       <c r="E51" t="inlineStr">
         <is>
           <t xml:space="preserve">Farda straight vermicelli, made from wheat.
-Pack size: 140 g.</t>
+Pack size: 140 g.
+Uses: sweet and savoury recipes.</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -5457,7 +5518,8 @@
       <c r="E52" t="inlineStr">
         <is>
           <t xml:space="preserve">Farda U-shaped vermicelli, made from wheat.
-Pack size: 130 g.</t>
+Pack size: 130 g.
+Uses: sweet and savoury recipes.</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">

</xml_diff>

<commit_message>
Polish supplied Farda Tea and Seran catalogs under Rule 804
</commit_message>
<xml_diff>
--- a/catalog-files/Farda_Foods_Professional.xlsx
+++ b/catalog-files/Farda_Foods_Professional.xlsx
@@ -2645,7 +2645,8 @@
       <c r="E12" t="inlineStr">
         <is>
           <t xml:space="preserve">Farda Himalayan pink salt for everyday seasoning.
-Pack size: 800 g.</t>
+Pack size: 800 g.
+Iodized pink salt sourced from Himalayan salt mines.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -2717,7 +2718,8 @@
         <is>
           <t xml:space="preserve">Farda straight vermicelli, made from wheat.
 Pack size: 350 g.
-Uses: sweet and savoury recipes.</t>
+Uses: sweet and savoury recipes.
+Smooth-textured wheat vermicelli with a delicate bite, designed to absorb the flavours of sweet or savoury dishes.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -3074,7 +3076,8 @@
       <c r="E18" t="inlineStr">
         <is>
           <t xml:space="preserve">Farda Chaat Masala is a spice blend for chaat and savoury snacks.
-Available pack sizes: 50 g, 100 g.</t>
+Available pack sizes: 50 g, 100 g.
+Flavour profile: tangy, spicy and savoury; suitable for snacks and street-food dishes.</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -3150,7 +3153,8 @@
       <c r="E19" t="inlineStr">
         <is>
           <t xml:space="preserve">Farda cumin powder, made from ground cumin seeds, for cooking and spice blends.
-Pack size: 50 g.</t>
+Pack size: 50 g.
+Suitable for Pakistani, Indian and other cuisines.</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -3434,7 +3438,8 @@
       <c r="E23" t="inlineStr">
         <is>
           <t xml:space="preserve">Farda red chilli powder for adding chilli flavour to food.
-Available pack sizes: 100 g, 200 g.</t>
+Available pack sizes: 100 g, 200 g.
+Made from hand-picked, sun-dried red chilli peppers, with a rich, smoky flavour.</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -3653,7 +3658,8 @@
         <is>
           <t xml:space="preserve">Farda Garam Masala Saabit is a whole-spice blend for Pakistani cooking.
 Pack size: 100 g.
-Ingredients (as listed): cloves, cinnamon, cardamoms, cumin, coriander, nutmeg, bay leaf, mace and black pepper.</t>
+Ingredients (as listed): cloves, cinnamon, cardamoms, cumin, coriander, nutmeg, bay leaf, mace and black pepper.
+The whole spices can be toasted and ground to release their aroma, producing a warm, mildly spicy seasoning.</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -3795,7 +3801,8 @@
       <c r="E28" t="inlineStr">
         <is>
           <t xml:space="preserve">Farda Chaat Masala Powder is a spice blend for chaat and savoury snacks.
-Pack quantity: 12.</t>
+Pack quantity: 12.
+Flavour profile: tangy, spicy and savoury; suitable for snacks and street-food dishes.</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -3938,7 +3945,8 @@
       <c r="E30" t="inlineStr">
         <is>
           <t xml:space="preserve">Farda red chilli powder for adding chilli flavour to food.
-Pack quantity: 12.</t>
+Pack quantity: 12.
+Made from hand-picked, sun-dried red chilli peppers, with a rich, smoky flavour.</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -4300,7 +4308,8 @@
         <is>
           <t xml:space="preserve">Farda Qorma Masala is a spice blend for qorma.
 Pack quantity: 12.
-Unit weight: 12 g.</t>
+Unit weight: 12 g.
+Flavour profile: warm, mellow spices with a subtle sweetness and an aromatic finish.</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4591,7 +4600,8 @@
         <is>
           <t xml:space="preserve">Farda Qorma Masala is a spice blend for qorma.
 Pack quantity: 12.
-Unit weight: 21 g.</t>
+Unit weight: 21 g.
+Flavour profile: warm, mellow spices with a subtle sweetness and an aromatic finish.</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -4806,7 +4816,8 @@
       <c r="E42" t="inlineStr">
         <is>
           <t xml:space="preserve">Farda Chicken Tikka Masala is a spice blend for chicken tikka.
-Pack size: 50 g.</t>
+Pack size: 50 g.
+A rich, tangy seasoning for marinated chicken or paneer.</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -5020,7 +5031,8 @@
       <c r="E45" t="inlineStr">
         <is>
           <t xml:space="preserve">Farda Qorma Masala is a spice blend for qorma.
-Pack size: 50 g.</t>
+Pack size: 50 g.
+Flavour profile: smoky, tangy and spicy; intended for seasoning marinated meat for qorma.</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -5091,7 +5103,8 @@
       <c r="E46" t="inlineStr">
         <is>
           <t xml:space="preserve">Farda Seekh Kabab Masala is a spice blend for seekh kababs.
-Pack size: 50 g.</t>
+Pack size: 50 g.
+Savoury, smoky seasoning for marinated minced meat used in seekh kababs.</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -5162,7 +5175,8 @@
       <c r="E47" t="inlineStr">
         <is>
           <t xml:space="preserve">Farda refined white salt, fortified with iodine, for everyday seasoning.
-Pack size: 800 g.</t>
+Pack size: 800 g.
+Fine white crystals with a neutral taste; refined to remove impurities and fortified with iodine.</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -5447,7 +5461,8 @@
         <is>
           <t xml:space="preserve">Farda straight vermicelli, made from wheat.
 Pack size: 140 g.
-Uses: sweet and savoury recipes.</t>
+Uses: sweet and savoury recipes.
+Smooth-textured wheat vermicelli with a delicate bite, designed to absorb the flavours of sweet or savoury dishes.</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -5519,7 +5534,8 @@
         <is>
           <t xml:space="preserve">Farda U-shaped vermicelli, made from wheat.
 Pack size: 130 g.
-Uses: sweet and savoury recipes.</t>
+Uses: sweet and savoury recipes.
+Smooth-textured wheat vermicelli with a delicate bite, designed to absorb the flavours of sweet or savoury dishes.</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">

</xml_diff>